<commit_message>
Account for the new blank row before each child sheet's header in the alt template
Organization_Template_Alternate.xlsx now has a blank row inserted
before the header row on every sheet except "How to use this
workbook" and "Main Org record" (Alt names, Addresses, Phones,
Emails, URLs, Contact people, Interfaces, Vendor info, Accounts,
External note). AlternateTemplateFlattener::flatten() had every one of
those sheets hardcoded to headerRow=1; updated all of them to
headerRow=2 so headers are still read from the right row instead of
the new blank one.

tests/fixtures/template_fixture_alt.xlsx gets the same blank row
inserted on every affected sheet, so the test fixture's layout matches
the real template and actually exercises the new header-row offset
rather than continuing to pass against the old layout.
</commit_message>
<xml_diff>
--- a/tests/fixtures/template_fixture_alt.xlsx
+++ b/tests/fixtures/template_fixture_alt.xlsx
@@ -686,80 +686,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A2:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="45" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="27" t="inlineStr">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>PAYMENT METHOD</t>
         </is>
       </c>
-      <c r="C1" s="27" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>CURRENCIES</t>
         </is>
       </c>
-      <c r="D1" s="27" t="inlineStr">
+      <c r="D2" s="27" t="inlineStr">
         <is>
           <t>CLAIMING INTERVAL</t>
         </is>
       </c>
-      <c r="E1" s="27" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>DISCOUNT %</t>
         </is>
       </c>
-      <c r="F1" s="27" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>EXP ACTIVATION INTERVAL</t>
         </is>
       </c>
-      <c r="G1" s="27" t="inlineStr">
+      <c r="G2" s="27" t="inlineStr">
         <is>
           <t>EXP INVOICE INTERVAL</t>
         </is>
       </c>
-      <c r="H1" s="27" t="inlineStr">
+      <c r="H2" s="27" t="inlineStr">
         <is>
           <t>EXP RECEIPT INTERVAL</t>
         </is>
       </c>
-      <c r="I1" s="27" t="inlineStr">
+      <c r="I2" s="27" t="inlineStr">
         <is>
           <t>RENEWAL ACTIVATION INTERVAL</t>
         </is>
       </c>
-      <c r="J1" s="27" t="inlineStr">
+      <c r="J2" s="27" t="inlineStr">
         <is>
           <t>SUBSCRIPTION INTERVAL</t>
         </is>
       </c>
-      <c r="K1" s="27" t="inlineStr">
+      <c r="K2" s="27" t="inlineStr">
         <is>
           <t>EXPORT TO ACCOUNTING (Y/)</t>
         </is>
       </c>
-      <c r="L1" s="27" t="inlineStr">
+      <c r="L2" s="27" t="inlineStr">
         <is>
           <t>TAX ID</t>
         </is>
       </c>
-      <c r="M1" s="27" t="inlineStr">
+      <c r="M2" s="27" t="inlineStr">
         <is>
           <t>TAX %</t>
         </is>
       </c>
-      <c r="N1" s="27" t="inlineStr">
+      <c r="N2" s="27" t="inlineStr">
         <is>
           <t>LIABLE FOR VAT (Y/N)</t>
         </is>
@@ -776,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A2:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.28515625" customWidth="1" style="20" min="1" max="1"/>
@@ -789,97 +790,98 @@
     <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="24">
-      <c r="A1" s="29" t="inlineStr">
+    <row r="1" customFormat="1" s="24"/>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="22" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>ACCOUNT NAME</t>
         </is>
       </c>
-      <c r="C1" s="30" t="inlineStr">
+      <c r="C2" s="30" t="inlineStr">
         <is>
           <t>ACCOUNT NUMBER</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>ACCOUNTING CODE</t>
         </is>
       </c>
-      <c r="F1" s="23" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>PAYMENT METHOD</t>
         </is>
       </c>
-      <c r="G1" s="30" t="inlineStr">
+      <c r="G2" s="30" t="inlineStr">
         <is>
           <t>ACCOUNT STATUS</t>
         </is>
       </c>
-      <c r="H1" s="26" t="inlineStr">
+      <c r="H2" s="26" t="inlineStr">
         <is>
           <t>LIBRARY EDI CODE</t>
         </is>
       </c>
-      <c r="I1" s="23" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>ACME</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Main Account</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
-      <c r="D2" s="18" t="n"/>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>SYS1</t>
         </is>
       </c>
-      <c r="F2" s="18" t="n"/>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H2" s="25" t="n"/>
-      <c r="I2" t="inlineStr">
+      <c r="H3" s="25" t="n"/>
+      <c r="I3" t="inlineStr">
         <is>
           <t>acct note</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="25" t="n"/>
+    <row r="4">
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="10" t="n"/>
+      <c r="C4" s="25" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -892,7 +894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A2:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.57" customWidth="1" min="1" max="1"/>
@@ -901,47 +903,26 @@
     <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="31" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="31" t="inlineStr">
+      <c r="B2" s="31" t="inlineStr">
         <is>
           <t>NOTE TYPE</t>
         </is>
       </c>
-      <c r="C1" s="31" t="inlineStr">
+      <c r="C2" s="31" t="inlineStr">
         <is>
           <t>NOTE TITLE</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>CONTENTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ACME</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>first note</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>first note body</t>
         </is>
       </c>
     </row>
@@ -953,10 +934,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>first note</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>first note body</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ACME</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>second note</t>
         </is>
@@ -1106,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A2:C5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="7.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.42578125" customWidth="1" min="1" max="1"/>
@@ -1114,32 +1117,21 @@
     <col width="13.28515625" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>ALT NAME</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ACME</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>AcmeAlias</t>
         </is>
       </c>
     </row>
@@ -1151,12 +1143,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Acme Corp</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Formal name</t>
+          <t>AcmeAlias</t>
         </is>
       </c>
     </row>
@@ -1167,6 +1154,23 @@
         </is>
       </c>
       <c r="B4" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Formal name</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ACME</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Acme Inc</t>
         </is>
@@ -1183,7 +1187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A2:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.28515625" customWidth="1" min="1" max="1"/>
@@ -1192,87 +1196,51 @@
     <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ADDR1 </t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>ADDR2</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CITY</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>REGION</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>POSTAL CODE</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>COUNTRY</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="I1" s="28" t="inlineStr">
+      <c r="I2" s="28" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ACME</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1 Main St</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>62701</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1284,10 +1252,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>1 Main St</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>62701</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ACME</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>2 Warehouse Rd</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
@@ -1309,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A2:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.7109375" customWidth="1" min="1" max="1"/>
@@ -1318,49 +1323,31 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>PHONE</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>ACME</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>555-1000</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1372,28 +1359,47 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
+          <t>555-1000</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>ACME</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
           <t>555-2000</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Fax</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="D4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ACME</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>555-3000</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
@@ -1418,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A2:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.140625" customWidth="1" min="1" max="1"/>
@@ -1428,47 +1434,31 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>ACME</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>info@acme.example</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1479,6 +1469,23 @@
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>info@acme.example</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>ACME</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>sales@acme.example</t>
         </is>
@@ -1500,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A2:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.140625" customWidth="1" min="1" max="1"/>
@@ -1510,67 +1517,35 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="31" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="31" t="inlineStr">
+      <c r="B2" s="31" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="C1" s="28" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="F1" s="28" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ACME</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://acme.example</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Main website</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>vendor note</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1582,10 +1557,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>https://acme.example</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Main website</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>vendor note</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ACME</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>https://support.acme.example</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>second url note</t>
         </is>
@@ -1607,7 +1614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A2:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="20.25" customHeight="1"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1621,104 +1628,105 @@
     <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customFormat="1" customHeight="1" s="3">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="20.25" customFormat="1" customHeight="1" s="3"/>
+    <row r="2" ht="20.25" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>LAST NAME</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>FIRST NAME</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>TITLE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PHONE </t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="3" ht="20.25" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>ACME</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Smith</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Jo</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>a note</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>jo@acme.example</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>555-4000</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>main contact</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="5" t="n"/>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="10" t="n"/>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1731,7 +1739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A2:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1743,98 +1751,99 @@
     <col width="13.140625" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>DELIVERY METHOD</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>USERNAME</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>PASSWORD</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>ACME</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Acme Admin</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>https://admin.acme.example</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" t="inlineStr">
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" t="inlineStr">
         <is>
           <t>iface note</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="10" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>